<commit_message>
Verdict all 104 quilt annotations against the data
61 aligned, 16 not, 27 unverifiable. Adds the per-action tab.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rh5PmZC78Sk962vrzXHy9F
</commit_message>
<xml_diff>
--- a/drafts/SLQS_action_check_09Sep2026.xlsx
+++ b/drafts/SLQS_action_check_09Sep2026.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="campaign pauses vs data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="target pauses vs data" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unmarked but same test" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="every action verdicted" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2834,7 +2835,6 @@
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>no orders past the click line</t>
@@ -2859,7 +2859,6 @@
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>no orders past the click line</t>
@@ -2938,7 +2937,6 @@
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>no orders past the click line</t>
@@ -2963,10 +2961,4233 @@
       <c r="E14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>no orders past the click line</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J105"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>campaign</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>your_action</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>clicks_7d</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>spend_7d</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>orders_7d</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cost_per_order</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SL-QS - navy quilt king - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F2" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>$28.98 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SL-QS - green quilt queen - [Quilt|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-SAGE-GREEN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>placement Placement Product Page 20% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>16 clicks, no orders — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SL-QS - green quilt queen - [Quilt|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-SAGE-GREEN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F4" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>$33.39 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SL-QS - king size bedspread - [Bedspread|King] - Broad - Disc - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>placement Placement Product Page 10% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>106</v>
+      </c>
+      <c r="F5" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>106 clicks, $24.31 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread king size - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F6" t="n">
+        <v>41.59</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>22 clicks, $20.80 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SL-QS - king size bedspread - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>placement Placement Top 20% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>11 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-COVERLET</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>39</v>
+      </c>
+      <c r="F8" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>$20.33 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SL-QS - king white quilt - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>22</v>
+      </c>
+      <c r="F9" t="n">
+        <v>28.24</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>22 clicks, no orders — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SL-QS - ivory quilt queen - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-IVORY</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>placement Placement Top 10% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>11</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>11 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-QUEEN-G</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>converting at $11.27, inside the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-COMP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>19</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>converting at $9.94, inside the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-CORE</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>62</v>
+      </c>
+      <c r="F13" t="n">
+        <v>32</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>32</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>$32.00 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread queen - [Bedspread|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>placement Placement Top 10% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>14</v>
+      </c>
+      <c r="F14" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>14 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-KING-G</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>placement Placement Rest Of Search 30% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>203</v>
+      </c>
+      <c r="F15" t="n">
+        <v>112.56</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>56.28</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>203 clicks, $56.28 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SL-QS - king size bedspread - [Bedspread|King] - Broad - Disc - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>placement Placement Rest Of Search 10% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>237</v>
+      </c>
+      <c r="F16" t="n">
+        <v>168.71</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>42.18</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>237 clicks, $42.18 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>placement Placement Product Page 20% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>397</v>
+      </c>
+      <c r="F17" t="n">
+        <v>321.59</v>
+      </c>
+      <c r="G17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" t="n">
+        <v>29.24</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>397 clicks, $29.24 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D-QS-SP-PHRASE-CATCH ALL-TWIN-G</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>53</v>
+      </c>
+      <c r="F18" t="n">
+        <v>54.05</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>53 clicks, no orders — past the line with nothing to show</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-B</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>56</v>
+      </c>
+      <c r="F19" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>$29.02 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SL-QS - B0DJ6WWZP2  - PAT - MS - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>33</v>
+      </c>
+      <c r="F20" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>$37.82 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-SUBS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>58</v>
+      </c>
+      <c r="F21" t="n">
+        <v>29.63</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>29.63</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>$29.63 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-SUBS</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" t="n">
+        <v>23.47</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>23.47</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>$23.47 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread king size - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>39</v>
+      </c>
+      <c r="F23" t="n">
+        <v>65.41</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>$32.70 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SL-QS - quilt set king size - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>53</v>
+      </c>
+      <c r="F24" t="n">
+        <v>44.93</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>22.47</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>$22.47 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-A</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>king bedspreads</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>pause keyword</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>68</v>
+      </c>
+      <c r="F25" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>$35.28 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-A</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>32</v>
+      </c>
+      <c r="F26" t="n">
+        <v>16.76</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>16.76</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>$16.76 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SL-QS - king quilt bedding set - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>23</v>
+      </c>
+      <c r="F27" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>23 clicks, no orders — past the line with nothing to show</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-BROAD-XCAT-ES</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>41</v>
+      </c>
+      <c r="F28" t="n">
+        <v>21.13</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>21.13</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>$21.13 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-BROAD-XCAT-ES</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>28</v>
+      </c>
+      <c r="F29" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>$14.66 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-KING-G</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Product Targeting</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>loose-match</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>pause product targeting</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>197</v>
+      </c>
+      <c r="F30" t="n">
+        <v>112.49</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>56.24</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>$56.24 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SL-QS - ivory quilt king - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-IVORY</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>10</v>
+      </c>
+      <c r="F31" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>10 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-KING-G</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>37</v>
+      </c>
+      <c r="F32" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>21.05</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>$21.05 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>oversize king bedspread</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>pause keyword</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>76</v>
+      </c>
+      <c r="F33" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="n">
+        <v>39.24</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>$39.24 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>76</v>
+      </c>
+      <c r="F34" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>39.24</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>$39.24 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>76</v>
+      </c>
+      <c r="F35" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>39.24</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>$39.24 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-BROAD-SIZE</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>bedding queen size</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>pause keyword</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>34</v>
+      </c>
+      <c r="F36" t="n">
+        <v>17.36</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>17.36</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>$17.36 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1441</v>
+      </c>
+      <c r="F37" t="n">
+        <v>979.64</v>
+      </c>
+      <c r="G37" t="n">
+        <v>61</v>
+      </c>
+      <c r="H37" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PAT-CONQUEST</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>111</v>
+      </c>
+      <c r="F38" t="n">
+        <v>65.20999999999999</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H38" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-A</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>163</v>
+      </c>
+      <c r="F39" t="n">
+        <v>84.78</v>
+      </c>
+      <c r="G39" t="n">
+        <v>5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread king - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>35</v>
+      </c>
+      <c r="F40" t="n">
+        <v>63.57</v>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-BROAD-SIZE</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>152</v>
+      </c>
+      <c r="F41" t="n">
+        <v>78.56999999999999</v>
+      </c>
+      <c r="G41" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-B</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>107</v>
+      </c>
+      <c r="F42" t="n">
+        <v>55.46</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" t="n">
+        <v>13.87</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-BROAD-XCAT-ES</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>189</v>
+      </c>
+      <c r="F43" t="n">
+        <v>96.95999999999999</v>
+      </c>
+      <c r="G43" t="n">
+        <v>7</v>
+      </c>
+      <c r="H43" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SL-QS - quilt king - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>29</v>
+      </c>
+      <c r="F44" t="n">
+        <v>40.08</v>
+      </c>
+      <c r="G44" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" t="n">
+        <v>13.36</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SL-QS - queen size bedspread - [Bedspread|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>22</v>
+      </c>
+      <c r="F45" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="n">
+        <v>13.71</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-COLOUR</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>60</v>
+      </c>
+      <c r="F46" t="n">
+        <v>30.98</v>
+      </c>
+      <c r="G46" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-COMP</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>40</v>
+      </c>
+      <c r="F47" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-EXACT-CLEARANCE</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>90</v>
+      </c>
+      <c r="F48" t="n">
+        <v>46.66</v>
+      </c>
+      <c r="G48" t="n">
+        <v>4</v>
+      </c>
+      <c r="H48" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-LOOSE</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>151</v>
+      </c>
+      <c r="F49" t="n">
+        <v>78.14</v>
+      </c>
+      <c r="G49" t="n">
+        <v>7</v>
+      </c>
+      <c r="H49" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SL-QS - B0BGS9VP2S- PAT - MS - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>31</v>
+      </c>
+      <c r="F50" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2</v>
+      </c>
+      <c r="H50" t="n">
+        <v>12.32</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-QUEEN-G</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>173</v>
+      </c>
+      <c r="F51" t="n">
+        <v>48.37</v>
+      </c>
+      <c r="G51" t="n">
+        <v>5</v>
+      </c>
+      <c r="H51" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-EXACT-PROVEN</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>30</v>
+      </c>
+      <c r="F52" t="n">
+        <v>15.54</v>
+      </c>
+      <c r="G52" t="n">
+        <v>2</v>
+      </c>
+      <c r="H52" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-XCAT</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>184</v>
+      </c>
+      <c r="F53" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="G53" t="n">
+        <v>12</v>
+      </c>
+      <c r="H53" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>D-QS-SP-PHRASE-(LTSF+TESTING)-SL-QUILT-SET-QUEEN-IVORY-queen quilt bedding</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>21</v>
+      </c>
+      <c r="F54" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>D-QS-SP-BROAD MODIFIER-(LTSF+TESTING)-SL-QUILT-SET-KING-LIGHT-GREY-lightweight king quilt</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>15</v>
+      </c>
+      <c r="F55" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SL-QS - queen size quilt bedding set - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>6</v>
+      </c>
+      <c r="F56" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>SL-QS - queen quilt sets with shams - [Quilt|Queen|Shams] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-WHITE</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>9</v>
+      </c>
+      <c r="F57" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>SL-QS - king quilts - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>18</v>
+      </c>
+      <c r="F58" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>SL-QS - lightweight queen quilts - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>4</v>
+      </c>
+      <c r="F59" t="n">
+        <v>7</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2</v>
+      </c>
+      <c r="H59" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>SL-QS - lightweight bedspreads queen size - [Bedspread|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-EXACT-king light weight quilt-Quilt|King-SL-QUILT-SET-KING-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-EXACT-lightweight bedspread-Bedspread-SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>SL-Quilt Sets-SP-Exact-Ranking-Fixed- SL-QUILT-SET-QUEEN-SAGE-GREEN-B0FGZZRZML-G</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>remove from negation</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>CANNOT VERIFY</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>marked on an Ad Group row with no keyword named, so there is no term to check against the search-term report — tell me which term each one refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>SL-QS-TESTING-NEW-FEATURE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>254</v>
+      </c>
+      <c r="F64" t="n">
+        <v>110.69</v>
+      </c>
+      <c r="G64" t="n">
+        <v>6</v>
+      </c>
+      <c r="H64" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>$18.45 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>101</v>
+      </c>
+      <c r="F65" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="G65" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>$24.13 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>SL-QS-TESTING-NEW-FEATURE</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>106</v>
+      </c>
+      <c r="F66" t="n">
+        <v>56.78</v>
+      </c>
+      <c r="G66" t="n">
+        <v>3</v>
+      </c>
+      <c r="H66" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>106 clicks, $18.93 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SL-QS - king size bedspread - [Bedspread|King] - Broad - Disc - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>placement Placement Top 10% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>150</v>
+      </c>
+      <c r="F67" t="n">
+        <v>122.44</v>
+      </c>
+      <c r="G67" t="n">
+        <v>6</v>
+      </c>
+      <c r="H67" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>150 clicks, $20.41 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>placement Placement Top 30% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>36</v>
+      </c>
+      <c r="F68" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="G68" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>36 clicks, $19.99 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>206</v>
+      </c>
+      <c r="F69" t="n">
+        <v>165.37</v>
+      </c>
+      <c r="G69" t="n">
+        <v>7</v>
+      </c>
+      <c r="H69" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>$23.62 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SL-QS-BROAD-LTSF-SL-QUILT-SET-QUEEN-TAUPE-lightweight quilts queen size</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>placement Placement Product Page 20% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>110</v>
+      </c>
+      <c r="F70" t="n">
+        <v>83.92</v>
+      </c>
+      <c r="G70" t="n">
+        <v>5</v>
+      </c>
+      <c r="H70" t="n">
+        <v>16.78</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>110 clicks, $16.78 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SL-QS - grey quilt queen size - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>12</v>
+      </c>
+      <c r="F71" t="n">
+        <v>17.38</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="n">
+        <v>17.38</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>12 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>SL-QS - green quilt queen - [Quilt|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-SAGE-GREEN</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>15</v>
+      </c>
+      <c r="F72" t="n">
+        <v>15.53</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" t="n">
+        <v>15.53</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>15 clicks, $15.53 per order — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SL-QS - queen size bed spread - [Bedspread|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-WHITE</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>placement Placement Rest Of Search 30% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>12</v>
+      </c>
+      <c r="F73" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" t="n">
+        <v>16.21</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>12 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>SL-QS - grey quilt queen size - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>13</v>
+      </c>
+      <c r="F74" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>13 clicks is below the 15-click line and it converted once at $18.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>placement Placement Top 30% -&gt; 20%</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>357</v>
+      </c>
+      <c r="F75" t="n">
+        <v>278.04</v>
+      </c>
+      <c r="G75" t="n">
+        <v>19</v>
+      </c>
+      <c r="H75" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>premium held at 20% on a placement at $14.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SL-QS-TESTING-NEW-FEATURE</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>254</v>
+      </c>
+      <c r="F76" t="n">
+        <v>110.69</v>
+      </c>
+      <c r="G76" t="n">
+        <v>6</v>
+      </c>
+      <c r="H76" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>$18.45 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-QUEEN-CATCH ALL</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>placement Placement Rest Of Search 30% -&gt; 20%</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>687</v>
+      </c>
+      <c r="F77" t="n">
+        <v>380.01</v>
+      </c>
+      <c r="G77" t="n">
+        <v>31</v>
+      </c>
+      <c r="H77" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>kept a premium on a placement converting at $12.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SL-QS - navy blue quilt queen - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 30%</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>10</v>
+      </c>
+      <c r="F78" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>10 clicks at this placement is below the line</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-AUTO-SUBS</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>151</v>
+      </c>
+      <c r="F79" t="n">
+        <v>78.31</v>
+      </c>
+      <c r="G79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H79" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>$19.58 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SL-QS-BROAD-LTSF-SL-QUILT-SET-QUEEN-TAUPE-lightweight quilts queen size</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>150</v>
+      </c>
+      <c r="F80" t="n">
+        <v>110.24</v>
+      </c>
+      <c r="G80" t="n">
+        <v>6</v>
+      </c>
+      <c r="H80" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>$18.37 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SL-QS - queen size bed spread - [Bedspread|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-WHITE</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>44</v>
+      </c>
+      <c r="F81" t="n">
+        <v>62.46</v>
+      </c>
+      <c r="G81" t="n">
+        <v>3</v>
+      </c>
+      <c r="H81" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>$20.82 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread king - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 30%</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>30</v>
+      </c>
+      <c r="F82" t="n">
+        <v>56.09</v>
+      </c>
+      <c r="G82" t="n">
+        <v>4</v>
+      </c>
+      <c r="H82" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>premium held at 30% on a placement at $14.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SL-QS - quilt set king size - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>53</v>
+      </c>
+      <c r="F83" t="n">
+        <v>44.93</v>
+      </c>
+      <c r="G83" t="n">
+        <v>2</v>
+      </c>
+      <c r="H83" t="n">
+        <v>22.46</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>$22.46 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SL-QS - white quilt king size - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>45</v>
+      </c>
+      <c r="F84" t="n">
+        <v>47.62</v>
+      </c>
+      <c r="G84" t="n">
+        <v>2</v>
+      </c>
+      <c r="H84" t="n">
+        <v>23.81</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>$23.81 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SL-QS - white king quilt - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>25</v>
+      </c>
+      <c r="F85" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>$24.85 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SL-QS - navy quilt king - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>35</v>
+      </c>
+      <c r="F86" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="G86" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" t="n">
+        <v>28.98</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>$28.98 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SL-QS - B0DJ6WWZP2  - PAT - MS - DO - SL-QUILT-SET-QUEEN-NAVY-BLUE</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>33</v>
+      </c>
+      <c r="F87" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="G87" t="n">
+        <v>1</v>
+      </c>
+      <c r="H87" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>$37.82 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>SL-QS - bedspread king size - [Bedspread|King] - Exact - Ran - DO - SL-QUILT-SET-KING-BLACK</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>39</v>
+      </c>
+      <c r="F88" t="n">
+        <v>65.41</v>
+      </c>
+      <c r="G88" t="n">
+        <v>2</v>
+      </c>
+      <c r="H88" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>$32.70 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>SL-QS - green quilt queen - [Quilt|Queen] - Phrase - Conv - DO - SL-QUILT-SET-QUEEN-SAGE-GREEN</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>35</v>
+      </c>
+      <c r="F89" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>$33.39 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SL-QS - king quilts for the bed - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>54</v>
+      </c>
+      <c r="F90" t="n">
+        <v>39.01</v>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" t="n">
+        <v>39.01</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>$39.01 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>76</v>
+      </c>
+      <c r="F91" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2</v>
+      </c>
+      <c r="H91" t="n">
+        <v>39.24</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>$39.24 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-COVERLET</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>72</v>
+      </c>
+      <c r="F92" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>$37.30 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-KING-G</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>230</v>
+      </c>
+      <c r="F93" t="n">
+        <v>119.88</v>
+      </c>
+      <c r="G93" t="n">
+        <v>2</v>
+      </c>
+      <c r="H93" t="n">
+        <v>59.94</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>$59.94 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-CORE</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Ad Group</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>pause ad group</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>97</v>
+      </c>
+      <c r="F94" t="n">
+        <v>50.25</v>
+      </c>
+      <c r="G94" t="n">
+        <v>1</v>
+      </c>
+      <c r="H94" t="n">
+        <v>50.25</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>$50.25 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>D-QS-SP-AUTO-QUEEN-G</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>24</v>
+      </c>
+      <c r="F95" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>24 clicks, no orders — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SL-QS-SP-PHRASE-SIZE-B</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>bed spread queen size</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>reduce bid</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>21</v>
+      </c>
+      <c r="F96" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>converting at $11.08, inside the cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SL-QS - grey quilt queen size - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>grey quilt queen size</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>pause keyword</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>13</v>
+      </c>
+      <c r="F97" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>13 clicks is below the 15-click line and it converted once at $18.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>SL-QS - oversize king bedspread - [Bedspread|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>placement Placement Rest Of Search 20% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>20</v>
+      </c>
+      <c r="F98" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>20 clicks, no orders — the premium is not earning</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>SL-QS - grey quilt queen size - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>pause product ad</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>13</v>
+      </c>
+      <c r="F99" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="G99" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>13 clicks is below the 15-click line and it converted once at $18.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>SL-QS - grey quilt queen size - [Quilt|Queen] - Exact - Ran - DO - SL-QUILT-SET-QUEEN-LIGHT-GREY</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>13</v>
+      </c>
+      <c r="F100" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="G100" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>NOT ALIGNED</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>13 clicks is below the 15-click line and it converted once at $18.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>D-QS-SP-BROAD MODIFIER-(LTSF+TESTING)- SL-QUILT-SET-KING-WHITE-G</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>26</v>
+      </c>
+      <c r="F101" t="n">
+        <v>8.66</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>26 clicks, no orders — past the line with nothing to show</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>SL-QS - king white quilt - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>27</v>
+      </c>
+      <c r="F102" t="n">
+        <v>32.69</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>27 clicks, no orders — past the line with nothing to show</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>SL-QS - king quilts for the bed - [Quilt|King] - Phrase - Conv - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>54</v>
+      </c>
+      <c r="F103" t="n">
+        <v>39.01</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+      <c r="H103" t="n">
+        <v>39.01</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>$39.01 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>SL-QS - white quilt king size - [Quilt|King] - Exact - Ran - DO - SL-QUILT-SET-KING-WHITE</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>pause campaign</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>45</v>
+      </c>
+      <c r="F104" t="n">
+        <v>47.62</v>
+      </c>
+      <c r="G104" t="n">
+        <v>2</v>
+      </c>
+      <c r="H104" t="n">
+        <v>23.81</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>$23.81 per order against the $13.20 cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>D-QS-SP-PHRASE-CATCH ALL-TWIN-G</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>placement Placement Top 50% -&gt; 0%</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>36</v>
+      </c>
+      <c r="F105" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>aligned</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>36 clicks, no orders — the premium is not earning</t>
         </is>
       </c>
     </row>

</xml_diff>